<commit_message>
fix(tabtools): close review findings and follow-ups, bump to 2.1.12
regtab: AIC/BIC/QICu count e(rank) again (base levels, mlogit base
equation and constraints excluded, matching estat ic), falling back to
the nonzero-SE coefficient count only when a cluster/replication/panel
cap binds. bs/bstrap/jknife prefixes are classified by level name, the
user's collect result labels are restored exactly, xtgee follows glm's
family/link rule, a covariate sharing its model's ancillary name shows
both rows, CI levels print without floating-point noise, and methods
nouns cover hetprobit, qreg and ivregress.

Every command passes title()/footnote() text through without macro
expansion, regtab/effecttab validate csv() before writing, the Markdown
writer escapes ~, and effecttab from() headers read 95% CI / p-value.
Adds regression suites for the follow-ups and the review fixes.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_regtab.xlsx
+++ b/tabtools/demo/demo_regtab.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="916" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="916" uniqueCount="232">
   <si>
     <t>Table 2. Propensity Score Model (Logistic Regression)</t>
   </si>
@@ -492,13 +492,10 @@
     <t>Base mean model</t>
   </si>
   <si>
-    <t>0.06</t>
-  </si>
-  <si>
-    <t>-0.13</t>
-  </si>
-  <si>
-    <t>-0.57</t>
+    <t>0.88</t>
+  </si>
+  <si>
+    <t>0.56</t>
   </si>
   <si>
     <t>26,200</t>
@@ -510,16 +507,16 @@
     <t>27142.20</t>
   </si>
   <si>
-    <t>(0.01, 0.01)</t>
-  </si>
-  <si>
-    <t>(0.04, 0.08)</t>
-  </si>
-  <si>
-    <t>(-0.22, -0.03)</t>
-  </si>
-  <si>
-    <t>(-0.67, -0.48)</t>
+    <t>(1.01, 1.01)</t>
+  </si>
+  <si>
+    <t>(1.04, 1.09)</t>
+  </si>
+  <si>
+    <t>(0.80, 0.97)</t>
+  </si>
+  <si>
+    <t>(0.51, 0.62)</t>
   </si>
   <si>
     <t>0.009</t>
@@ -528,31 +525,31 @@
     <t>Adjusted mean model</t>
   </si>
   <si>
-    <t>0.08</t>
-  </si>
-  <si>
-    <t>-0.06</t>
-  </si>
-  <si>
-    <t>-0.72</t>
-  </si>
-  <si>
-    <t>0.80</t>
+    <t>1.08</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>0.49</t>
+  </si>
+  <si>
+    <t>2.23</t>
   </si>
   <si>
     <t>26596.04</t>
   </si>
   <si>
-    <t>(0.06, 0.10)</t>
-  </si>
-  <si>
-    <t>(-0.15, 0.04)</t>
-  </si>
-  <si>
-    <t>(-0.82, -0.62)</t>
-  </si>
-  <si>
-    <t>(0.68, 0.93)</t>
+    <t>(1.06, 1.11)</t>
+  </si>
+  <si>
+    <t>(0.86, 1.04)</t>
+  </si>
+  <si>
+    <t>(0.44, 0.54)</t>
+  </si>
+  <si>
+    <t>(1.97, 2.53)</t>
   </si>
   <si>
     <t>0.26</t>
@@ -640,9 +637,6 @@
   </si>
   <si>
     <t>0.007</t>
-  </si>
-  <si>
-    <t>0.88</t>
   </si>
   <si>
     <t>0.39</t>
@@ -1513,7 +1507,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="12" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>1</v>
@@ -1536,7 +1530,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="62" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D2" s="61" t="s">
         <v>1</v>
@@ -1573,10 +1567,10 @@
         <v>137</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E4" s="70" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5">
@@ -1590,10 +1584,10 @@
         <v>14</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6">
@@ -1610,7 +1604,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7">
@@ -1658,10 +1652,10 @@
         <v>78</v>
       </c>
       <c r="D9" s="70" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10">
@@ -1675,10 +1669,10 @@
         <v>78</v>
       </c>
       <c r="D10" s="70" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11">
@@ -1686,7 +1680,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>1</v>
@@ -1703,7 +1697,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="69" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C12" s="71" t="s">
         <v>16</v>
@@ -1720,16 +1714,16 @@
         <v>1</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14">
@@ -1737,16 +1731,16 @@
         <v>1</v>
       </c>
       <c r="B14" s="69" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D14" s="70" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15">
@@ -1754,16 +1748,16 @@
         <v>1</v>
       </c>
       <c r="B15" s="69" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C15" s="70" t="s">
         <v>38</v>
       </c>
       <c r="D15" s="70" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="16">
@@ -1777,10 +1771,10 @@
         <v>20</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17">
@@ -1794,10 +1788,10 @@
         <v>15</v>
       </c>
       <c r="D17" s="70" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>205</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18">
@@ -1808,10 +1802,10 @@
         <v>10</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E18" s="16" t="s">
         <v>94</v>
@@ -1828,10 +1822,10 @@
         <v>137</v>
       </c>
       <c r="D19" s="73" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E19" s="73" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -1858,7 +1852,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>1</v>
@@ -1881,7 +1875,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
@@ -1918,10 +1912,10 @@
         <v>137</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5">
@@ -1932,13 +1926,13 @@
         <v>2</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E5" s="44" t="s">
         <v>209</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="E5" s="44" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="6">
@@ -1955,7 +1949,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
@@ -1966,18 +1960,18 @@
         <v>8</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E7" s="47" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="78" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
@@ -2006,7 +2000,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="12" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>1</v>
@@ -2029,7 +2023,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
@@ -2066,10 +2060,10 @@
         <v>137</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5">
@@ -2117,10 +2111,10 @@
         <v>20</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8">
@@ -2137,7 +2131,7 @@
         <v>24</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9">
@@ -2148,10 +2142,10 @@
         <v>10</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E9" s="44" t="s">
         <v>94</v>
@@ -2168,15 +2162,15 @@
         <v>137</v>
       </c>
       <c r="D10" s="46" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E10" s="47" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="78" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C11" s="0"/>
       <c r="D11" s="0"/>
@@ -2206,7 +2200,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="12" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>1</v>
@@ -2229,7 +2223,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
@@ -2266,10 +2260,10 @@
         <v>137</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5">
@@ -2280,13 +2274,13 @@
         <v>2</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6">
@@ -2303,7 +2297,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7">
@@ -2314,13 +2308,13 @@
         <v>8</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8">
@@ -2334,10 +2328,10 @@
         <v>19</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9">
@@ -2345,10 +2339,10 @@
         <v>1</v>
       </c>
       <c r="B9" s="48" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C9" s="52" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D9" s="51" t="s">
         <v>1</v>
@@ -2362,10 +2356,10 @@
         <v>1</v>
       </c>
       <c r="B10" s="43" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D10" s="46" t="s">
         <v>1</v>
@@ -2376,7 +2370,7 @@
     </row>
     <row r="11">
       <c r="B11" s="78" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C11" s="0"/>
       <c r="D11" s="0"/>
@@ -4345,10 +4339,10 @@
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
     <col min="2" max="2" width="24.7109375" style="1" customWidth="true"/>
     <col min="3" max="3" width="8.2109375" style="1" customWidth="true"/>
-    <col min="4" max="4" width="14.2109375" style="1" customWidth="true"/>
+    <col min="4" max="4" width="12.2109375" style="1" customWidth="true"/>
     <col min="5" max="5" width="7.7109375" style="1" customWidth="true"/>
     <col min="6" max="6" width="8.2109375" style="1" customWidth="true"/>
-    <col min="7" max="7" width="14.2109375" style="1" customWidth="true"/>
+    <col min="7" max="7" width="12.2109375" style="1" customWidth="true"/>
     <col min="8" max="8" width="7.7109375" style="1" customWidth="true"/>
   </cols>
   <sheetData>
@@ -4395,7 +4389,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>1</v>
@@ -4412,7 +4406,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>104</v>
+        <v>13</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>22</v>
@@ -4421,7 +4415,7 @@
         <v>31</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>104</v>
+        <v>13</v>
       </c>
       <c r="G3" s="31" t="s">
         <v>22</v>
@@ -4438,19 +4432,19 @@
         <v>148</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>105</v>
+        <v>19</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E4" s="44" t="s">
         <v>94</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>105</v>
+        <v>19</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H4" s="44" t="s">
         <v>94</v>
@@ -4464,19 +4458,19 @@
         <v>149</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>94</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H5" s="44" t="s">
         <v>94</v>
@@ -4490,22 +4484,22 @@
         <v>150</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H6" s="44" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">
@@ -4516,19 +4510,19 @@
         <v>151</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>94</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H7" s="44" t="s">
         <v>94</v>
@@ -4551,10 +4545,10 @@
         <v>1</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H8" s="44" t="s">
         <v>94</v>
@@ -4568,7 +4562,7 @@
         <v>54</v>
       </c>
       <c r="C9" s="52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D9" s="51" t="s">
         <v>1</v>
@@ -4577,7 +4571,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G9" s="51" t="s">
         <v>1</v>
@@ -4594,7 +4588,7 @@
         <v>101</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>1</v>
@@ -4603,7 +4597,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>1</v>
@@ -4620,7 +4614,7 @@
         <v>153</v>
       </c>
       <c r="C11" s="53" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D11" s="46" t="s">
         <v>1</v>
@@ -4629,7 +4623,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="53" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G11" s="46" t="s">
         <v>1</v>

</xml_diff>